<commit_message>
Update House PTR data (2026-10-17)
</commit_message>
<xml_diff>
--- a/data/03_verification/House_PTR_Verification_2026.xlsx
+++ b/data/03_verification/House_PTR_Verification_2026.xlsx
@@ -48736,7 +48736,7 @@
       </c>
       <c r="K1092" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>needs_fallback</t>
         </is>
       </c>
     </row>
@@ -59473,7 +59473,7 @@
       </c>
       <c r="K1329" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -72250,7 +72250,7 @@
       </c>
       <c r="K1618" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -79416,7 +79416,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
@@ -79426,7 +79426,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -79452,7 +79452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79826,6 +79826,13 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>9116378</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update House PTR data (2026-10-24)
</commit_message>
<xml_diff>
--- a/data/03_verification/House_PTR_Verification_2026.xlsx
+++ b/data/03_verification/House_PTR_Verification_2026.xlsx
@@ -24621,7 +24621,7 @@
       </c>
       <c r="K549" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -37203,7 +37203,7 @@
       </c>
       <c r="K835" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -80252,7 +80252,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>